<commit_message>
Golden Cala Shoof API Deploymnet on Sandbox
</commit_message>
<xml_diff>
--- a/Golden Cala/Scripts/Shoof Integration/Item/Technical Reference.xlsx
+++ b/Golden Cala/Scripts/Shoof Integration/Item/Technical Reference.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NetSuiteCompanies\Golden Cala\Scripts\Shoof Integration\Item\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A4017B-4F6D-4784-9838-B896DD7E5B0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{915AC685-7193-4CDF-A030-2A4C184C1CF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3375" yWindow="3375" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t>Type</t>
   </si>
@@ -73,6 +73,12 @@
   </si>
   <si>
     <t>Product Color</t>
+  </si>
+  <si>
+    <t>SKU Code</t>
+  </si>
+  <si>
+    <t>custitem_vs_sku</t>
   </si>
 </sst>
 </file>
@@ -410,7 +416,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="2" bestFit="1" customWidth="1"/>
@@ -489,6 +495,20 @@
         <v>13</v>
       </c>
     </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>